<commit_message>
Add batch script to set up and run Holy War environment
- Created 'Avvia Holy War.bat' to automate the setup of a Python virtual environment.
- Checks for Python installation and creates a virtual environment if not present.
- Installs required dependencies using pip if they are not already installed.
- Launches the Holy War application with specified JSON configuration.
- Includes error handling for setup and execution failures.
</commit_message>
<xml_diff>
--- a/Holy War.xlsx
+++ b/Holy War.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\admin\Documents\Holy-War-Python-Test\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Tech\Documents\Holy-War-Python-Test\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE26190D-A4A0-4628-A4A3-CD03F60687DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12BF4CF0-7D40-4E49-AC5D-F100009DEF2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1035" yWindow="2565" windowWidth="21600" windowHeight="10140" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1560" yWindow="1560" windowWidth="21600" windowHeight="11295" firstSheet="2" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Foglio1" sheetId="1" r:id="rId1"/>
@@ -1962,9 +1962,6 @@
     <t>Ah Puch</t>
   </si>
   <si>
-    <t>Ogni volta che un Token o un Santo viene mandato dal campo al cimitero, questo santo riceve +1 Fede e +1 Forza.</t>
-  </si>
-  <si>
     <t>Anima Errante</t>
   </si>
   <si>
@@ -2275,6 +2272,9 @@
   </si>
   <si>
     <t>Finche questa carta + sul terreno, ogni tuo santo ottiene +3 forza per ogni Ba Xian presente sul tuo terreno e +3 fede per ogni Ba Xian nel tuo cimitero.</t>
+  </si>
+  <si>
+    <t>Ogni volta che un Santo viene mandato dal campo al cimitero, questo santo riceve +1 Fede e +1 Forza.</t>
   </si>
 </sst>
 </file>
@@ -2385,7 +2385,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2469,17 +2469,11 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -7844,7 +7838,7 @@
         <v>6</v>
       </c>
       <c r="H1" s="27" t="s">
-        <v>744</v>
+        <v>743</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
@@ -7862,7 +7856,7 @@
       </c>
       <c r="E2" s="23"/>
       <c r="F2" s="24" t="s">
-        <v>742</v>
+        <v>741</v>
       </c>
       <c r="G2" s="26" t="s">
         <v>10</v>
@@ -7946,7 +7940,7 @@
       </c>
       <c r="E6" s="23"/>
       <c r="F6" s="24" t="s">
-        <v>740</v>
+        <v>739</v>
       </c>
       <c r="G6" s="26" t="s">
         <v>10</v>
@@ -8054,7 +8048,7 @@
       <c r="D11" s="23"/>
       <c r="E11" s="23"/>
       <c r="F11" s="24" t="s">
-        <v>732</v>
+        <v>731</v>
       </c>
       <c r="G11" s="26" t="s">
         <v>10</v>
@@ -8118,7 +8112,7 @@
       <c r="D14" s="23"/>
       <c r="E14" s="23"/>
       <c r="F14" s="24" t="s">
-        <v>747</v>
+        <v>746</v>
       </c>
       <c r="G14" s="26" t="s">
         <v>10</v>
@@ -8184,7 +8178,7 @@
       </c>
       <c r="E17" s="23"/>
       <c r="F17" s="24" t="s">
-        <v>743</v>
+        <v>742</v>
       </c>
       <c r="G17" s="26" t="s">
         <v>10</v>
@@ -8204,7 +8198,7 @@
       <c r="D18" s="23"/>
       <c r="E18" s="23"/>
       <c r="F18" s="24" t="s">
-        <v>737</v>
+        <v>736</v>
       </c>
       <c r="G18" s="26" t="s">
         <v>10</v>
@@ -8252,7 +8246,7 @@
         <v>2</v>
       </c>
       <c r="F20" s="24" t="s">
-        <v>746</v>
+        <v>745</v>
       </c>
       <c r="G20" s="26" t="s">
         <v>10</v>
@@ -8378,7 +8372,7 @@
         <v>8</v>
       </c>
       <c r="F25" s="24" t="s">
-        <v>745</v>
+        <v>744</v>
       </c>
       <c r="G25" s="26" t="s">
         <v>10</v>
@@ -8516,7 +8510,7 @@
       </c>
       <c r="E31" s="23"/>
       <c r="F31" s="24" t="s">
-        <v>748</v>
+        <v>747</v>
       </c>
       <c r="G31" s="26" t="s">
         <v>10</v>
@@ -8572,15 +8566,15 @@
       <c r="B34" s="29" t="s">
         <v>12</v>
       </c>
-      <c r="C34" s="30">
+      <c r="C34" s="28">
         <v>4</v>
       </c>
-      <c r="D34" s="30"/>
-      <c r="E34" s="30"/>
-      <c r="F34" s="31" t="s">
-        <v>735</v>
-      </c>
-      <c r="G34" s="32" t="s">
+      <c r="D34" s="28"/>
+      <c r="E34" s="28"/>
+      <c r="F34" s="30" t="s">
+        <v>734</v>
+      </c>
+      <c r="G34" s="7" t="s">
         <v>10</v>
       </c>
       <c r="H34" s="28"/>
@@ -8592,15 +8586,15 @@
       <c r="B35" s="29" t="s">
         <v>12</v>
       </c>
-      <c r="C35" s="30">
+      <c r="C35" s="28">
         <v>4</v>
       </c>
-      <c r="D35" s="30"/>
-      <c r="E35" s="30"/>
-      <c r="F35" s="31" t="s">
-        <v>733</v>
-      </c>
-      <c r="G35" s="32" t="s">
+      <c r="D35" s="28"/>
+      <c r="E35" s="28"/>
+      <c r="F35" s="30" t="s">
+        <v>732</v>
+      </c>
+      <c r="G35" s="7" t="s">
         <v>10</v>
       </c>
       <c r="H35" s="28"/>
@@ -8612,15 +8606,15 @@
       <c r="B36" s="29" t="s">
         <v>12</v>
       </c>
-      <c r="C36" s="30">
+      <c r="C36" s="28">
         <v>5</v>
       </c>
-      <c r="D36" s="30"/>
-      <c r="E36" s="30"/>
-      <c r="F36" s="31" t="s">
+      <c r="D36" s="28"/>
+      <c r="E36" s="28"/>
+      <c r="F36" s="30" t="s">
         <v>25</v>
       </c>
-      <c r="G36" s="32" t="s">
+      <c r="G36" s="7" t="s">
         <v>10</v>
       </c>
       <c r="H36" s="28"/>
@@ -8632,15 +8626,15 @@
       <c r="B37" s="29" t="s">
         <v>12</v>
       </c>
-      <c r="C37" s="30">
+      <c r="C37" s="28">
         <v>3</v>
       </c>
-      <c r="D37" s="30"/>
-      <c r="E37" s="30"/>
-      <c r="F37" s="31" t="s">
-        <v>734</v>
-      </c>
-      <c r="G37" s="32" t="s">
+      <c r="D37" s="28"/>
+      <c r="E37" s="28"/>
+      <c r="F37" s="30" t="s">
+        <v>733</v>
+      </c>
+      <c r="G37" s="7" t="s">
         <v>10</v>
       </c>
       <c r="H37" s="28"/>
@@ -8652,15 +8646,15 @@
       <c r="B38" s="29" t="s">
         <v>12</v>
       </c>
-      <c r="C38" s="30">
+      <c r="C38" s="28">
         <v>2</v>
       </c>
-      <c r="D38" s="30"/>
-      <c r="E38" s="30"/>
-      <c r="F38" s="31" t="s">
+      <c r="D38" s="28"/>
+      <c r="E38" s="28"/>
+      <c r="F38" s="30" t="s">
         <v>13</v>
       </c>
-      <c r="G38" s="32" t="s">
+      <c r="G38" s="7" t="s">
         <v>10</v>
       </c>
       <c r="H38" s="28"/>
@@ -8672,15 +8666,15 @@
       <c r="B39" s="29" t="s">
         <v>31</v>
       </c>
-      <c r="C39" s="30">
+      <c r="C39" s="28">
         <v>3</v>
       </c>
-      <c r="D39" s="30"/>
-      <c r="E39" s="30"/>
-      <c r="F39" s="31" t="s">
-        <v>738</v>
-      </c>
-      <c r="G39" s="32" t="s">
+      <c r="D39" s="28"/>
+      <c r="E39" s="28"/>
+      <c r="F39" s="30" t="s">
+        <v>737</v>
+      </c>
+      <c r="G39" s="7" t="s">
         <v>10</v>
       </c>
       <c r="H39" s="28"/>
@@ -8692,15 +8686,15 @@
       <c r="B40" s="29" t="s">
         <v>31</v>
       </c>
-      <c r="C40" s="30">
+      <c r="C40" s="28">
         <v>4</v>
       </c>
-      <c r="D40" s="30"/>
-      <c r="E40" s="30"/>
-      <c r="F40" s="31" t="s">
+      <c r="D40" s="28"/>
+      <c r="E40" s="28"/>
+      <c r="F40" s="30" t="s">
         <v>32</v>
       </c>
-      <c r="G40" s="32" t="s">
+      <c r="G40" s="7" t="s">
         <v>10</v>
       </c>
       <c r="H40" s="28"/>
@@ -8758,7 +8752,7 @@
       <c r="D43" s="23"/>
       <c r="E43" s="23"/>
       <c r="F43" s="24" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
       <c r="G43" s="26" t="s">
         <v>10</v>
@@ -8802,7 +8796,7 @@
       </c>
       <c r="E45" s="23"/>
       <c r="F45" s="24" t="s">
-        <v>741</v>
+        <v>740</v>
       </c>
       <c r="G45" s="26" t="s">
         <v>10</v>
@@ -8912,7 +8906,7 @@
       </c>
       <c r="E50" s="23"/>
       <c r="F50" s="24" t="s">
-        <v>739</v>
+        <v>738</v>
       </c>
       <c r="G50" s="26" t="s">
         <v>10</v>
@@ -21200,7 +21194,7 @@
         <v>7</v>
       </c>
       <c r="F2" s="12" t="s">
-        <v>644</v>
+        <v>748</v>
       </c>
       <c r="G2" s="11" t="s">
         <v>140</v>
@@ -21208,7 +21202,7 @@
     </row>
     <row r="3" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="12" t="s">
-        <v>645</v>
+        <v>644</v>
       </c>
       <c r="B3" s="12" t="s">
         <v>59</v>
@@ -21223,7 +21217,7 @@
         <v>3</v>
       </c>
       <c r="F3" s="12" t="s">
-        <v>646</v>
+        <v>645</v>
       </c>
       <c r="G3" s="11" t="s">
         <v>140</v>
@@ -21231,7 +21225,7 @@
     </row>
     <row r="4" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
-        <v>647</v>
+        <v>646</v>
       </c>
       <c r="B4" s="12" t="s">
         <v>8</v>
@@ -21244,7 +21238,7 @@
       </c>
       <c r="E4" s="14"/>
       <c r="F4" s="12" t="s">
-        <v>648</v>
+        <v>647</v>
       </c>
       <c r="G4" s="11" t="s">
         <v>140</v>
@@ -21252,7 +21246,7 @@
     </row>
     <row r="5" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="12" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
       <c r="B5" s="12" t="s">
         <v>59</v>
@@ -21267,7 +21261,7 @@
         <v>6</v>
       </c>
       <c r="F5" s="12" t="s">
-        <v>650</v>
+        <v>649</v>
       </c>
       <c r="G5" s="11" t="s">
         <v>140</v>
@@ -21275,7 +21269,7 @@
     </row>
     <row r="6" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="12" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
       <c r="B6" s="12" t="s">
         <v>8</v>
@@ -21288,7 +21282,7 @@
       </c>
       <c r="E6" s="14"/>
       <c r="F6" s="12" t="s">
-        <v>652</v>
+        <v>651</v>
       </c>
       <c r="G6" s="11" t="s">
         <v>140</v>
@@ -21296,7 +21290,7 @@
     </row>
     <row r="7" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="12" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
       <c r="B7" s="12" t="s">
         <v>8</v>
@@ -21309,7 +21303,7 @@
       </c>
       <c r="E7" s="14"/>
       <c r="F7" s="12" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="G7" s="11" t="s">
         <v>140</v>
@@ -21317,7 +21311,7 @@
     </row>
     <row r="8" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="12" t="s">
-        <v>655</v>
+        <v>654</v>
       </c>
       <c r="B8" s="12" t="s">
         <v>54</v>
@@ -21330,7 +21324,7 @@
       </c>
       <c r="E8" s="14"/>
       <c r="F8" s="12" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
       <c r="G8" s="11" t="s">
         <v>140</v>
@@ -21338,7 +21332,7 @@
     </row>
     <row r="9" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="12" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
       <c r="B9" s="12" t="s">
         <v>31</v>
@@ -21349,7 +21343,7 @@
       <c r="D9" s="14"/>
       <c r="E9" s="14"/>
       <c r="F9" s="12" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="G9" s="11" t="s">
         <v>140</v>
@@ -21357,7 +21351,7 @@
     </row>
     <row r="10" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="12" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="B10" s="12" t="s">
         <v>59</v>
@@ -21372,7 +21366,7 @@
         <v>6</v>
       </c>
       <c r="F10" s="12" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="G10" s="11" t="s">
         <v>140</v>
@@ -21380,7 +21374,7 @@
     </row>
     <row r="11" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="12" t="s">
-        <v>661</v>
+        <v>660</v>
       </c>
       <c r="B11" s="12" t="s">
         <v>59</v>
@@ -21395,7 +21389,7 @@
         <v>4</v>
       </c>
       <c r="F11" s="12" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="G11" s="11" t="s">
         <v>140</v>
@@ -21403,7 +21397,7 @@
     </row>
     <row r="12" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="12" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
       <c r="B12" s="12" t="s">
         <v>31</v>
@@ -21414,7 +21408,7 @@
       <c r="D12" s="14"/>
       <c r="E12" s="14"/>
       <c r="F12" s="12" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="G12" s="11" t="s">
         <v>140</v>
@@ -21422,7 +21416,7 @@
     </row>
     <row r="13" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="12" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="B13" s="12" t="s">
         <v>361</v>
@@ -21431,7 +21425,7 @@
       <c r="D13" s="14"/>
       <c r="E13" s="14"/>
       <c r="F13" s="12" t="s">
-        <v>666</v>
+        <v>665</v>
       </c>
       <c r="G13" s="11" t="s">
         <v>140</v>
@@ -21439,7 +21433,7 @@
     </row>
     <row r="14" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="12" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="B14" s="12" t="s">
         <v>12</v>
@@ -21450,7 +21444,7 @@
       <c r="D14" s="14"/>
       <c r="E14" s="14"/>
       <c r="F14" s="12" t="s">
-        <v>668</v>
+        <v>667</v>
       </c>
       <c r="G14" s="11" t="s">
         <v>140</v>
@@ -21458,7 +21452,7 @@
     </row>
     <row r="15" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="12" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
       <c r="B15" s="12" t="s">
         <v>12</v>
@@ -21469,7 +21463,7 @@
       <c r="D15" s="14"/>
       <c r="E15" s="14"/>
       <c r="F15" s="12" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="G15" s="11" t="s">
         <v>140</v>
@@ -21477,7 +21471,7 @@
     </row>
     <row r="16" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="12" t="s">
-        <v>671</v>
+        <v>670</v>
       </c>
       <c r="B16" s="12" t="s">
         <v>12</v>
@@ -21488,7 +21482,7 @@
       <c r="D16" s="14"/>
       <c r="E16" s="14"/>
       <c r="F16" s="12" t="s">
-        <v>672</v>
+        <v>671</v>
       </c>
       <c r="G16" s="11" t="s">
         <v>140</v>
@@ -21496,7 +21490,7 @@
     </row>
     <row r="17" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="12" t="s">
-        <v>673</v>
+        <v>672</v>
       </c>
       <c r="B17" s="12" t="s">
         <v>31</v>
@@ -21507,7 +21501,7 @@
       <c r="D17" s="14"/>
       <c r="E17" s="14"/>
       <c r="F17" s="12" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
       <c r="G17" s="11" t="s">
         <v>140</v>
@@ -21515,7 +21509,7 @@
     </row>
     <row r="18" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="12" t="s">
-        <v>675</v>
+        <v>674</v>
       </c>
       <c r="B18" s="12" t="s">
         <v>12</v>
@@ -21526,7 +21520,7 @@
       <c r="D18" s="14"/>
       <c r="E18" s="14"/>
       <c r="F18" s="12" t="s">
-        <v>676</v>
+        <v>675</v>
       </c>
       <c r="G18" s="11" t="s">
         <v>140</v>
@@ -21534,7 +21528,7 @@
     </row>
     <row r="19" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="12" t="s">
-        <v>677</v>
+        <v>676</v>
       </c>
       <c r="B19" s="12" t="s">
         <v>59</v>
@@ -21549,7 +21543,7 @@
         <v>6</v>
       </c>
       <c r="F19" s="12" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
       <c r="G19" s="11" t="s">
         <v>140</v>
@@ -21557,7 +21551,7 @@
     </row>
     <row r="20" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="12" t="s">
-        <v>679</v>
+        <v>678</v>
       </c>
       <c r="B20" s="12" t="s">
         <v>8</v>
@@ -21570,7 +21564,7 @@
       </c>
       <c r="E20" s="14"/>
       <c r="F20" s="12" t="s">
-        <v>680</v>
+        <v>679</v>
       </c>
       <c r="G20" s="11" t="s">
         <v>140</v>
@@ -21578,7 +21572,7 @@
     </row>
     <row r="21" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="12" t="s">
-        <v>681</v>
+        <v>680</v>
       </c>
       <c r="B21" s="12" t="s">
         <v>450</v>
@@ -21599,7 +21593,7 @@
     </row>
     <row r="22" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="12" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
       <c r="B22" s="12" t="s">
         <v>31</v>
@@ -21610,7 +21604,7 @@
       <c r="D22" s="14"/>
       <c r="E22" s="14"/>
       <c r="F22" s="12" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
       <c r="G22" s="11" t="s">
         <v>140</v>
@@ -21618,7 +21612,7 @@
     </row>
     <row r="23" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="12" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
       <c r="B23" s="12" t="s">
         <v>54</v>
@@ -21631,7 +21625,7 @@
       </c>
       <c r="E23" s="14"/>
       <c r="F23" s="12" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
       <c r="G23" s="11" t="s">
         <v>140</v>
@@ -21639,7 +21633,7 @@
     </row>
     <row r="24" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="12" t="s">
-        <v>686</v>
+        <v>685</v>
       </c>
       <c r="B24" s="12" t="s">
         <v>59</v>
@@ -21654,7 +21648,7 @@
         <v>5</v>
       </c>
       <c r="F24" s="12" t="s">
-        <v>687</v>
+        <v>686</v>
       </c>
       <c r="G24" s="11" t="s">
         <v>140</v>
@@ -21662,7 +21656,7 @@
     </row>
     <row r="25" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="12" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
       <c r="B25" s="12" t="s">
         <v>8</v>
@@ -21675,7 +21669,7 @@
       </c>
       <c r="E25" s="14"/>
       <c r="F25" s="12" t="s">
-        <v>689</v>
+        <v>688</v>
       </c>
       <c r="G25" s="11" t="s">
         <v>140</v>
@@ -24260,7 +24254,7 @@
     </row>
     <row r="2" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
-        <v>690</v>
+        <v>689</v>
       </c>
       <c r="B2" s="12" t="s">
         <v>12</v>
@@ -24271,7 +24265,7 @@
       <c r="D2" s="14"/>
       <c r="E2" s="14"/>
       <c r="F2" s="12" t="s">
-        <v>691</v>
+        <v>690</v>
       </c>
       <c r="G2" s="8" t="s">
         <v>145</v>
@@ -24279,7 +24273,7 @@
     </row>
     <row r="3" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
-        <v>692</v>
+        <v>691</v>
       </c>
       <c r="B3" s="12" t="s">
         <v>12</v>
@@ -24290,7 +24284,7 @@
       <c r="D3" s="14"/>
       <c r="E3" s="14"/>
       <c r="F3" s="12" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
       <c r="G3" s="8" t="s">
         <v>145</v>
@@ -24298,7 +24292,7 @@
     </row>
     <row r="4" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
       <c r="B4" s="12" t="s">
         <v>31</v>
@@ -24309,7 +24303,7 @@
       <c r="D4" s="14"/>
       <c r="E4" s="14"/>
       <c r="F4" s="12" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="G4" s="8" t="s">
         <v>145</v>
@@ -24317,7 +24311,7 @@
     </row>
     <row r="5" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
-        <v>696</v>
+        <v>695</v>
       </c>
       <c r="B5" s="12" t="s">
         <v>12</v>
@@ -24328,7 +24322,7 @@
       <c r="D5" s="14"/>
       <c r="E5" s="14"/>
       <c r="F5" s="12" t="s">
-        <v>697</v>
+        <v>696</v>
       </c>
       <c r="G5" s="8" t="s">
         <v>145</v>
@@ -24336,7 +24330,7 @@
     </row>
     <row r="6" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
-        <v>698</v>
+        <v>697</v>
       </c>
       <c r="B6" s="12" t="s">
         <v>12</v>
@@ -24347,7 +24341,7 @@
       <c r="D6" s="14"/>
       <c r="E6" s="14"/>
       <c r="F6" s="12" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
       <c r="G6" s="8" t="s">
         <v>145</v>
@@ -24355,7 +24349,7 @@
     </row>
     <row r="7" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
       <c r="B7" s="12" t="s">
         <v>31</v>
@@ -24366,7 +24360,7 @@
       <c r="D7" s="14"/>
       <c r="E7" s="14"/>
       <c r="F7" s="12" t="s">
-        <v>701</v>
+        <v>700</v>
       </c>
       <c r="G7" s="8" t="s">
         <v>145</v>
@@ -24374,7 +24368,7 @@
     </row>
     <row r="8" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="18" t="s">
-        <v>702</v>
+        <v>701</v>
       </c>
       <c r="B8" s="12" t="s">
         <v>12</v>
@@ -24385,7 +24379,7 @@
       <c r="D8" s="14"/>
       <c r="E8" s="14"/>
       <c r="F8" s="12" t="s">
-        <v>703</v>
+        <v>702</v>
       </c>
       <c r="G8" s="8" t="s">
         <v>145</v>
@@ -24393,7 +24387,7 @@
     </row>
     <row r="9" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="18" t="s">
-        <v>704</v>
+        <v>703</v>
       </c>
       <c r="B9" s="12" t="s">
         <v>12</v>
@@ -24404,7 +24398,7 @@
       <c r="D9" s="14"/>
       <c r="E9" s="14"/>
       <c r="F9" s="12" t="s">
-        <v>705</v>
+        <v>704</v>
       </c>
       <c r="G9" s="8" t="s">
         <v>145</v>
@@ -24412,7 +24406,7 @@
     </row>
     <row r="10" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="18" t="s">
-        <v>706</v>
+        <v>705</v>
       </c>
       <c r="B10" s="12" t="s">
         <v>12</v>
@@ -24423,7 +24417,7 @@
       <c r="D10" s="14"/>
       <c r="E10" s="14"/>
       <c r="F10" s="12" t="s">
-        <v>707</v>
+        <v>706</v>
       </c>
       <c r="G10" s="8" t="s">
         <v>145</v>
@@ -24431,7 +24425,7 @@
     </row>
     <row r="11" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="18" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="B11" s="12" t="s">
         <v>12</v>
@@ -24442,7 +24436,7 @@
       <c r="D11" s="14"/>
       <c r="E11" s="14"/>
       <c r="F11" s="12" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
       <c r="G11" s="8" t="s">
         <v>145</v>
@@ -24450,7 +24444,7 @@
     </row>
     <row r="12" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="18" t="s">
-        <v>710</v>
+        <v>709</v>
       </c>
       <c r="B12" s="12" t="s">
         <v>31</v>
@@ -24461,7 +24455,7 @@
       <c r="D12" s="14"/>
       <c r="E12" s="14"/>
       <c r="F12" s="12" t="s">
-        <v>711</v>
+        <v>710</v>
       </c>
       <c r="G12" s="8" t="s">
         <v>145</v>
@@ -24469,7 +24463,7 @@
     </row>
     <row r="13" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="18" t="s">
-        <v>712</v>
+        <v>711</v>
       </c>
       <c r="B13" s="12" t="s">
         <v>12</v>
@@ -24480,7 +24474,7 @@
       <c r="D13" s="14"/>
       <c r="E13" s="14"/>
       <c r="F13" s="12" t="s">
-        <v>713</v>
+        <v>712</v>
       </c>
       <c r="G13" s="8" t="s">
         <v>145</v>
@@ -24488,7 +24482,7 @@
     </row>
     <row r="14" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="18" t="s">
-        <v>714</v>
+        <v>713</v>
       </c>
       <c r="B14" s="12" t="s">
         <v>31</v>
@@ -24499,7 +24493,7 @@
       <c r="D14" s="14"/>
       <c r="E14" s="14"/>
       <c r="F14" s="12" t="s">
-        <v>715</v>
+        <v>714</v>
       </c>
       <c r="G14" s="8" t="s">
         <v>145</v>
@@ -24507,7 +24501,7 @@
     </row>
     <row r="15" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
-        <v>716</v>
+        <v>715</v>
       </c>
       <c r="B15" s="12" t="s">
         <v>12</v>
@@ -24518,7 +24512,7 @@
       <c r="D15" s="14"/>
       <c r="E15" s="14"/>
       <c r="F15" s="12" t="s">
-        <v>717</v>
+        <v>716</v>
       </c>
       <c r="G15" s="8" t="s">
         <v>145</v>
@@ -24526,7 +24520,7 @@
     </row>
     <row r="16" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
       <c r="B16" s="12" t="s">
         <v>12</v>
@@ -24537,7 +24531,7 @@
       <c r="D16" s="14"/>
       <c r="E16" s="14"/>
       <c r="F16" s="12" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
       <c r="G16" s="8" t="s">
         <v>145</v>
@@ -24545,7 +24539,7 @@
     </row>
     <row r="17" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
-        <v>720</v>
+        <v>719</v>
       </c>
       <c r="B17" s="12" t="s">
         <v>12</v>
@@ -24556,7 +24550,7 @@
       <c r="D17" s="14"/>
       <c r="E17" s="14"/>
       <c r="F17" s="12" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
       <c r="G17" s="8" t="s">
         <v>145</v>
@@ -24564,7 +24558,7 @@
     </row>
     <row r="18" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="B18" s="12" t="s">
         <v>31</v>
@@ -24575,7 +24569,7 @@
       <c r="D18" s="14"/>
       <c r="E18" s="14"/>
       <c r="F18" s="12" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="G18" s="8" t="s">
         <v>145</v>
@@ -24583,7 +24577,7 @@
     </row>
     <row r="19" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
-        <v>724</v>
+        <v>723</v>
       </c>
       <c r="B19" s="12" t="s">
         <v>59</v>
@@ -24598,7 +24592,7 @@
         <v>2</v>
       </c>
       <c r="F19" s="12" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="G19" s="8" t="s">
         <v>145</v>
@@ -24606,7 +24600,7 @@
     </row>
     <row r="20" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
       <c r="B20" s="12" t="s">
         <v>31</v>
@@ -24617,7 +24611,7 @@
       <c r="D20" s="14"/>
       <c r="E20" s="14"/>
       <c r="F20" s="12" t="s">
-        <v>727</v>
+        <v>726</v>
       </c>
       <c r="G20" s="8" t="s">
         <v>145</v>
@@ -24625,7 +24619,7 @@
     </row>
     <row r="21" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
-        <v>728</v>
+        <v>727</v>
       </c>
       <c r="B21" s="12" t="s">
         <v>12</v>
@@ -24636,7 +24630,7 @@
       <c r="D21" s="14"/>
       <c r="E21" s="14"/>
       <c r="F21" s="12" t="s">
-        <v>729</v>
+        <v>728</v>
       </c>
       <c r="G21" s="8" t="s">
         <v>145</v>
@@ -24644,7 +24638,7 @@
     </row>
     <row r="22" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="18" t="s">
-        <v>730</v>
+        <v>729</v>
       </c>
       <c r="B22" s="12" t="s">
         <v>31</v>
@@ -24655,7 +24649,7 @@
       <c r="D22" s="14"/>
       <c r="E22" s="14"/>
       <c r="F22" s="12" t="s">
-        <v>731</v>
+        <v>730</v>
       </c>
       <c r="G22" s="8" t="s">
         <v>145</v>

</xml_diff>